<commit_message>
refactor: migrate test infrastructure from PostgreSQL to Firestore emulator and introduce fixture-based seeding.
</commit_message>
<xml_diff>
--- a/demo-output/DEMO - Otter Client 1 (Check-In)/AppointmentFlowSheet/DEMO - Otter Client 1 (Check-In) Appointment Flow Sheet.xlsx
+++ b/demo-output/DEMO - Otter Client 1 (Check-In)/AppointmentFlowSheet/DEMO - Otter Client 1 (Check-In) Appointment Flow Sheet.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="23">
   <si>
     <t>DATE</t>
   </si>
@@ -34,13 +34,13 @@
     <t xml:space="preserve">Virtual </t>
   </si>
   <si>
-    <t>July 13, 2026</t>
+    <t>July 31, 2026</t>
   </si>
   <si>
-    <t>BM:  good, healthy, solid</t>
+    <t>BM: I feel like I've been having really good poops. Great, good, healthy, solid</t>
   </si>
   <si>
-    <t>gallbladder pain — stones confirmed on ultrasound, surgeon wanted removal; yeast infections; headaches; hot at night</t>
+    <t>the environmental like stressors for everyone has been; my energy has been feeling pretty stable throughout the day; I drank caffeine too late, so I didn't want to sleep last night; I got one in July 4th again; I was definitely really stressed for a little bit</t>
   </si>
   <si>
     <t xml:space="preserve">LAYING 1 FOUNDATIONS:
@@ -54,9 +54,8 @@
 CNS:
 DENTAL: 
 HORMONAL: 
-ADDITIONAL:
-hypothalamus is a little bit offline
-nervous system's like definitely doing pretty well</t>
+ADDITIONAL: we found the hypothalamus is like a little bit offline
+we're just looking for zinc, though</t>
   </si>
   <si>
     <r>
@@ -260,12 +259,19 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Start zinc
+    <t xml:space="preserve">Continue Zinc
+Continue B complex
 Start Simplex F
-Start oregano</t>
+Start Oregano
+Stop ADHS
+Stop Wormwood
+Stop Vitamin D
+Stop Fish oil
+Continue Chlorella
+Continue Cataplexy</t>
   </si>
   <si>
-    <t>SLEEP:</t>
+    <t>SLEEP: I didn't want to sleep last night</t>
   </si>
   <si>
     <t>WATER:</t>
@@ -274,10 +280,10 @@
     <t>CYCLE:</t>
   </si>
   <si>
-    <t>EXERCISE: walking on the treadmill, 10-15 minutes</t>
+    <t>EXERCISE: I've just been trying to like get myself consistent in the gym</t>
   </si>
   <si>
-    <t>DIET: smoothies, eggs, trying to eat more protein</t>
+    <t>DIET: I have been tracking my like my macros and stuff</t>
   </si>
   <si>
     <t xml:space="preserve">BM: </t>
@@ -492,6 +498,9 @@
       </rPr>
       <t>:</t>
     </r>
+  </si>
+  <si>
+    <t>SLEEP:</t>
   </si>
   <si>
     <t>EXERCISE:</t>
@@ -1384,7 +1393,7 @@
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
@@ -1534,7 +1543,7 @@
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
@@ -1584,7 +1593,7 @@
     <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="15"/>
       <c r="B25" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
@@ -1726,7 +1735,7 @@
     <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>
       <c r="B30" s="9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
@@ -1876,7 +1885,7 @@
     <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="15"/>
       <c r="B36" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
@@ -1926,7 +1935,7 @@
     <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="15"/>
       <c r="B38" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C38" s="17"/>
       <c r="D38" s="17"/>
@@ -2068,7 +2077,7 @@
     <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" s="15"/>
       <c r="B43" s="9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C43" s="17"/>
       <c r="D43" s="17"/>
@@ -2218,7 +2227,7 @@
     <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" s="15"/>
       <c r="B49" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C49" s="17"/>
       <c r="D49" s="17"/>
@@ -2268,7 +2277,7 @@
     <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" s="15"/>
       <c r="B51" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C51" s="17"/>
       <c r="D51" s="17"/>
@@ -2410,7 +2419,7 @@
     <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" s="15"/>
       <c r="B56" s="9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C56" s="17"/>
       <c r="D56" s="17"/>
@@ -2560,7 +2569,7 @@
     <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A62" s="15"/>
       <c r="B62" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C62" s="17"/>
       <c r="D62" s="17"/>
@@ -2610,7 +2619,7 @@
     <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A64" s="15"/>
       <c r="B64" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C64" s="17"/>
       <c r="D64" s="17"/>
@@ -2752,7 +2761,7 @@
     <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" s="15"/>
       <c r="B69" s="9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C69" s="17"/>
       <c r="D69" s="17"/>
@@ -2902,7 +2911,7 @@
     <row r="75" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A75" s="15"/>
       <c r="B75" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C75" s="17"/>
       <c r="D75" s="17"/>
@@ -2952,7 +2961,7 @@
     <row r="77" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A77" s="15"/>
       <c r="B77" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C77" s="17"/>
       <c r="D77" s="17"/>
@@ -3094,7 +3103,7 @@
     <row r="82" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A82" s="15"/>
       <c r="B82" s="9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C82" s="17"/>
       <c r="D82" s="17"/>
@@ -3244,7 +3253,7 @@
     <row r="88" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A88" s="15"/>
       <c r="B88" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C88" s="17"/>
       <c r="D88" s="17"/>
@@ -3294,7 +3303,7 @@
     <row r="90" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A90" s="15"/>
       <c r="B90" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C90" s="17"/>
       <c r="D90" s="17"/>

</xml_diff>